<commit_message>
Version del proyecto al dia 18 de septiembre de 2026
</commit_message>
<xml_diff>
--- a/Archivos/CONFIGURACION/Config.xlsx
+++ b/Archivos/CONFIGURACION/Config.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Procesos_Uipath\541_DISPOINFOMEDALIABRYAM_NF_SEG_SEG\Archivos\CONFIGURACION\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81E24466-7028-4D63-9CA0-1D34DC724BB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{749633F2-C631-468A-8B17-80C0E90F42C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -867,7 +867,7 @@
     <t>1UVfEf_Rn2nx13Ursoj0rYL7qGP5-346SpHQL_z-_0VM</t>
   </si>
   <si>
-    <t>D</t>
+    <t>C</t>
   </si>
 </sst>
 </file>
@@ -1644,7 +1644,7 @@
       </c>
       <c r="B7" s="2" t="str">
         <f>_xlfn.CONCAT($E$3, ":\Procesos_UiPath\"&amp;B3&amp;"\Archivos\")</f>
-        <v>D:\Procesos_UiPath\541_DISPOINFOMEDALIABRYAM_NF_SEG_SEG\Archivos\</v>
+        <v>C:\Procesos_UiPath\541_DISPOINFOMEDALIABRYAM_NF_SEG_SEG\Archivos\</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>133</v>
@@ -1656,7 +1656,7 @@
       </c>
       <c r="B8" s="2" t="str">
         <f>_xlfn.CONCAT($E$3, ":\Procesos_UiPath\"&amp;B3&amp;"\Archivos\"&amp;B4&amp;"\")</f>
-        <v>D:\Procesos_UiPath\541_DISPOINFOMEDALIABRYAM_NF_SEG_SEG\Archivos\Temporal\</v>
+        <v>C:\Procesos_UiPath\541_DISPOINFOMEDALIABRYAM_NF_SEG_SEG\Archivos\Temporal\</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>134</v>
@@ -1668,7 +1668,7 @@
       </c>
       <c r="B9" s="2" t="str">
         <f>_xlfn.CONCAT($E$3, ":\Procesos_UiPath\"&amp;B3&amp;"\Archivos\"&amp;B4&amp;"_Error")</f>
-        <v>D:\Procesos_UiPath\541_DISPOINFOMEDALIABRYAM_NF_SEG_SEG\Archivos\Temporal_Error</v>
+        <v>C:\Procesos_UiPath\541_DISPOINFOMEDALIABRYAM_NF_SEG_SEG\Archivos\Temporal_Error</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>136</v>
@@ -1680,7 +1680,7 @@
       </c>
       <c r="B10" t="str">
         <f>_xlfn.CONCAT($E$3, ":\Procesos_UiPath\"&amp;B3&amp;"\Archivos\FORMATOS\")</f>
-        <v>D:\Procesos_UiPath\541_DISPOINFOMEDALIABRYAM_NF_SEG_SEG\Archivos\FORMATOS\</v>
+        <v>C:\Procesos_UiPath\541_DISPOINFOMEDALIABRYAM_NF_SEG_SEG\Archivos\FORMATOS\</v>
       </c>
       <c r="C10" t="s">
         <v>137</v>
@@ -1692,7 +1692,7 @@
       </c>
       <c r="B11" s="2" t="str">
         <f>_xlfn.CONCAT($E$3, ":\Procesos_UiPath\"&amp;B3&amp;"\Archivos\CONFIGURACION\")</f>
-        <v>D:\Procesos_UiPath\541_DISPOINFOMEDALIABRYAM_NF_SEG_SEG\Archivos\CONFIGURACION\</v>
+        <v>C:\Procesos_UiPath\541_DISPOINFOMEDALIABRYAM_NF_SEG_SEG\Archivos\CONFIGURACION\</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>139</v>
@@ -1704,7 +1704,7 @@
       </c>
       <c r="B12" s="2" t="str">
         <f>_xlfn.CONCAT($E$3, ":\Procesos_UiPath\"&amp;B3&amp;"\Archivos\Exceptions_Screenshots\")</f>
-        <v>D:\Procesos_UiPath\541_DISPOINFOMEDALIABRYAM_NF_SEG_SEG\Archivos\Exceptions_Screenshots\</v>
+        <v>C:\Procesos_UiPath\541_DISPOINFOMEDALIABRYAM_NF_SEG_SEG\Archivos\Exceptions_Screenshots\</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>141</v>
@@ -2351,7 +2351,7 @@
       </c>
       <c r="B88" s="41" t="str">
         <f>_xlfn.CONCAT(E3,":\Procesos_UiPath\Llaves\crp-pro-ccoe-automat-c9c501f57fdd_NF.json")</f>
-        <v>D:\Procesos_UiPath\Llaves\crp-pro-ccoe-automat-c9c501f57fdd_NF.json</v>
+        <v>C:\Procesos_UiPath\Llaves\crp-pro-ccoe-automat-c9c501f57fdd_NF.json</v>
       </c>
       <c r="C88" s="42" t="s">
         <v>124</v>

</xml_diff>

<commit_message>
Version del proyecto al 23 / 09 / 2026
</commit_message>
<xml_diff>
--- a/Archivos/CONFIGURACION/Config.xlsx
+++ b/Archivos/CONFIGURACION/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Procesos_Uipath\541_DISPOINFOMEDALIABRYAM_NF_SEG_SEG\Archivos\CONFIGURACION\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{749633F2-C631-468A-8B17-80C0E90F42C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCF54E17-520B-4EB5-9531-37F1E30055CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="243">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="254">
   <si>
     <t>Name</t>
   </si>
@@ -819,18 +819,6 @@
     <t>C:\Program Files\Python38\</t>
   </si>
   <si>
-    <t>MedalliaUser</t>
-  </si>
-  <si>
-    <t>MedalliaPassword</t>
-  </si>
-  <si>
-    <t>cricardov@liverpool.com.mx</t>
-  </si>
-  <si>
-    <t>3ras3_un4JM</t>
-  </si>
-  <si>
     <t>541_DISPOINFOMEDALIABRYAM_NF_SEG_SEG</t>
   </si>
   <si>
@@ -864,17 +852,62 @@
     <t>Template de Google Sheet de Suburbia</t>
   </si>
   <si>
-    <t>1UVfEf_Rn2nx13Ursoj0rYL7qGP5-346SpHQL_z-_0VM</t>
+    <t>Id_Sheet_PlantillaRegistrosGlobales</t>
+  </si>
+  <si>
+    <t>1Ho4_5n3e3SyFwS-abRHqeLuCXK__oC4Sz74XjNLceSk</t>
+  </si>
+  <si>
+    <t>Id_Sheet_FolderReportesDiarios</t>
+  </si>
+  <si>
+    <t>15dkrlT8OO6PJwchlXyckIVZmWdjoCbpE</t>
+  </si>
+  <si>
+    <t>Cred_Medallia</t>
+  </si>
+  <si>
+    <t>Usr_Active_Directory</t>
+  </si>
+  <si>
+    <t>Cred_Generica</t>
+  </si>
+  <si>
+    <t>IdSheetReprocesos</t>
+  </si>
+  <si>
+    <t>1LadTK_nCaO-3Den47XRLUp_ODoGlwgsBnScrscPbx0M</t>
+  </si>
+  <si>
+    <t>Archivo que determina las ejecuciones</t>
+  </si>
+  <si>
+    <t>IdSheetCorreosEnviados</t>
+  </si>
+  <si>
+    <t>1Bt8YI2hz2viYufv1tQpBy8gFyQR-RiKS</t>
+  </si>
+  <si>
+    <t>Folder para guardar historicos de correos enviados.</t>
+  </si>
+  <si>
+    <t>1aIFFCmYWICxlWv_rqnVRtiX2G4vyAWygaUnZZPSuwYE</t>
   </si>
   <si>
     <t>C</t>
+  </si>
+  <si>
+    <t>IdCarpetaReportes</t>
+  </si>
+  <si>
+    <t>1i32WDbFZOhjmaND-ySCiCkkLQsiXoBQr</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18">
+  <fonts count="19">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -987,6 +1020,12 @@
       <sz val="11"/>
       <color theme="10"/>
       <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -1109,7 +1148,7 @@
     <xf numFmtId="0" fontId="10" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1227,6 +1266,7 @@
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="3"/>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Accent2" xfId="2" builtinId="33"/>
@@ -1550,7 +1590,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z992"/>
+  <dimension ref="A1:Z993"/>
   <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="43.54296875" customWidth="1"/>
@@ -1601,13 +1641,13 @@
         <v>123</v>
       </c>
       <c r="B3" s="25" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="C3" s="26" t="s">
         <v>128</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>242</v>
+        <v>251</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1">
@@ -1632,10 +1672,10 @@
     </row>
     <row r="6" spans="1:26" ht="14.5">
       <c r="A6" s="2" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
     </row>
     <row r="7" spans="1:26" ht="14.25" customHeight="1">
@@ -2308,7 +2348,7 @@
         <v>102</v>
       </c>
       <c r="B84" s="39" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="C84" s="39" t="s">
         <v>172</v>
@@ -2316,32 +2356,32 @@
     </row>
     <row r="85" spans="1:3" ht="14.25" customHeight="1">
       <c r="A85" s="52" t="s">
+        <v>230</v>
+      </c>
+      <c r="B85" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="B85" s="2" t="s">
-        <v>238</v>
-      </c>
       <c r="C85" s="2" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
     </row>
     <row r="86" spans="1:3" ht="14.25" customHeight="1">
       <c r="A86" s="2" t="s">
-        <v>239</v>
-      </c>
-      <c r="B86" t="s">
-        <v>241</v>
+        <v>235</v>
+      </c>
+      <c r="B86" s="2" t="s">
+        <v>250</v>
       </c>
       <c r="C86" s="2" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
     </row>
     <row r="87" spans="1:3" ht="14.25" customHeight="1">
       <c r="A87" s="52" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="C87" s="2"/>
     </row>
@@ -2401,34 +2441,63 @@
       </c>
       <c r="C95" s="22"/>
     </row>
-    <row r="96" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="97" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="96" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A96" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="B96" s="2" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A97" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="B97" t="s">
+        <v>240</v>
+      </c>
+    </row>
     <row r="98" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A98" s="12"/>
-      <c r="B98" s="12"/>
-      <c r="C98" s="12"/>
-    </row>
-    <row r="99" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="100" spans="1:3" ht="14.25" customHeight="1"/>
+      <c r="A98" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="B98" t="s">
+        <v>245</v>
+      </c>
+      <c r="C98" s="2" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A99" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="B99" t="s">
+        <v>248</v>
+      </c>
+      <c r="C99" s="2" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A100" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="B100" t="s">
+        <v>253</v>
+      </c>
+    </row>
     <row r="101" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="102" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="103" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A103" s="2" t="s">
-        <v>226</v>
-      </c>
-      <c r="B103" s="51" t="s">
-        <v>228</v>
-      </c>
-    </row>
+    <row r="103" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="104" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A104" s="2" t="s">
-        <v>227</v>
-      </c>
-      <c r="B104" s="2" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="105" spans="1:3" ht="14.25" customHeight="1"/>
+      <c r="A104" s="2"/>
+      <c r="B104" s="51"/>
+    </row>
+    <row r="105" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A105" s="2"/>
+      <c r="B105" s="2"/>
+    </row>
     <row r="106" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="107" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="108" spans="1:3" ht="14.25" customHeight="1"/>
@@ -3316,13 +3385,11 @@
     <row r="990" ht="14.25" customHeight="1"/>
     <row r="991" ht="14.25" customHeight="1"/>
     <row r="992" ht="14.25" customHeight="1"/>
+    <row r="993" ht="14.25" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="3"/>
-  <hyperlinks>
-    <hyperlink ref="B103" r:id="rId1" xr:uid="{635E4254-AF21-4D23-80EB-9B5D00625052}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -5766,7 +5833,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="13.453125" bestFit="1" customWidth="1"/>
@@ -5803,6 +5870,22 @@
         <v>45</v>
       </c>
     </row>
+    <row r="3" spans="1:4">
+      <c r="A3" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="B3" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="B4" s="53" t="s">
+        <v>242</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Version del proyecto al dia 1 de octubre de 2026
</commit_message>
<xml_diff>
--- a/Archivos/CONFIGURACION/Config.xlsx
+++ b/Archivos/CONFIGURACION/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Procesos_Uipath\541_DISPOINFOMEDALIABRYAM_NF_SEG_SEG\Archivos\CONFIGURACION\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCF54E17-520B-4EB5-9531-37F1E30055CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BF18854-130B-4024-B638-4DD9C075DB85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -813,94 +813,94 @@
     <t>END POINTS PARA MODULO "CHAT_RPA"</t>
   </si>
   <si>
+    <t>C:\Program Files\Python38\</t>
+  </si>
+  <si>
+    <t>541_DISPOINFOMEDALIABRYAM_NF_SEG_SEG</t>
+  </si>
+  <si>
+    <t>Descargas</t>
+  </si>
+  <si>
+    <t>Downloads\</t>
+  </si>
+  <si>
+    <t>0AHVIhGN0elUOUk9PVA</t>
+  </si>
+  <si>
+    <t>Id_Template_Liverpool</t>
+  </si>
+  <si>
+    <t>Template de Google Sheet de Liverpool</t>
+  </si>
+  <si>
+    <t>Id_Carpeta_Config_Bot</t>
+  </si>
+  <si>
+    <t>1MW2qJxEnyfY3t5gfL9MOCKiYjNtK1CNp</t>
+  </si>
+  <si>
+    <t>1ZUrDKGkjrHELaHsYlGOsv9Sxd8xapjPZQoTOnLnCYZQ</t>
+  </si>
+  <si>
+    <t>Id_Template_Suburbia</t>
+  </si>
+  <si>
+    <t>Template de Google Sheet de Suburbia</t>
+  </si>
+  <si>
+    <t>Id_Sheet_PlantillaRegistrosGlobales</t>
+  </si>
+  <si>
+    <t>1Ho4_5n3e3SyFwS-abRHqeLuCXK__oC4Sz74XjNLceSk</t>
+  </si>
+  <si>
+    <t>Id_Sheet_FolderReportesDiarios</t>
+  </si>
+  <si>
+    <t>15dkrlT8OO6PJwchlXyckIVZmWdjoCbpE</t>
+  </si>
+  <si>
+    <t>Cred_Medallia</t>
+  </si>
+  <si>
+    <t>Usr_Active_Directory</t>
+  </si>
+  <si>
+    <t>Cred_Generica</t>
+  </si>
+  <si>
+    <t>IdSheetReprocesos</t>
+  </si>
+  <si>
+    <t>1LadTK_nCaO-3Den47XRLUp_ODoGlwgsBnScrscPbx0M</t>
+  </si>
+  <si>
+    <t>Archivo que determina las ejecuciones</t>
+  </si>
+  <si>
+    <t>IdSheetCorreosEnviados</t>
+  </si>
+  <si>
+    <t>1Bt8YI2hz2viYufv1tQpBy8gFyQR-RiKS</t>
+  </si>
+  <si>
+    <t>Folder para guardar historicos de correos enviados.</t>
+  </si>
+  <si>
+    <t>1aIFFCmYWICxlWv_rqnVRtiX2G4vyAWygaUnZZPSuwYE</t>
+  </si>
+  <si>
+    <t>IdCarpetaReportes</t>
+  </si>
+  <si>
+    <t>1i32WDbFZOhjmaND-ySCiCkkLQsiXoBQr</t>
+  </si>
+  <si>
     <t>C:\Users\USR\AppData\Local\Programs\Python\Python38\</t>
   </si>
   <si>
-    <t>C:\Program Files\Python38\</t>
-  </si>
-  <si>
-    <t>541_DISPOINFOMEDALIABRYAM_NF_SEG_SEG</t>
-  </si>
-  <si>
-    <t>Descargas</t>
-  </si>
-  <si>
-    <t>Downloads\</t>
-  </si>
-  <si>
-    <t>0AHVIhGN0elUOUk9PVA</t>
-  </si>
-  <si>
-    <t>Id_Template_Liverpool</t>
-  </si>
-  <si>
-    <t>Template de Google Sheet de Liverpool</t>
-  </si>
-  <si>
-    <t>Id_Carpeta_Config_Bot</t>
-  </si>
-  <si>
-    <t>1MW2qJxEnyfY3t5gfL9MOCKiYjNtK1CNp</t>
-  </si>
-  <si>
-    <t>1ZUrDKGkjrHELaHsYlGOsv9Sxd8xapjPZQoTOnLnCYZQ</t>
-  </si>
-  <si>
-    <t>Id_Template_Suburbia</t>
-  </si>
-  <si>
-    <t>Template de Google Sheet de Suburbia</t>
-  </si>
-  <si>
-    <t>Id_Sheet_PlantillaRegistrosGlobales</t>
-  </si>
-  <si>
-    <t>1Ho4_5n3e3SyFwS-abRHqeLuCXK__oC4Sz74XjNLceSk</t>
-  </si>
-  <si>
-    <t>Id_Sheet_FolderReportesDiarios</t>
-  </si>
-  <si>
-    <t>15dkrlT8OO6PJwchlXyckIVZmWdjoCbpE</t>
-  </si>
-  <si>
-    <t>Cred_Medallia</t>
-  </si>
-  <si>
-    <t>Usr_Active_Directory</t>
-  </si>
-  <si>
-    <t>Cred_Generica</t>
-  </si>
-  <si>
-    <t>IdSheetReprocesos</t>
-  </si>
-  <si>
-    <t>1LadTK_nCaO-3Den47XRLUp_ODoGlwgsBnScrscPbx0M</t>
-  </si>
-  <si>
-    <t>Archivo que determina las ejecuciones</t>
-  </si>
-  <si>
-    <t>IdSheetCorreosEnviados</t>
-  </si>
-  <si>
-    <t>1Bt8YI2hz2viYufv1tQpBy8gFyQR-RiKS</t>
-  </si>
-  <si>
-    <t>Folder para guardar historicos de correos enviados.</t>
-  </si>
-  <si>
-    <t>1aIFFCmYWICxlWv_rqnVRtiX2G4vyAWygaUnZZPSuwYE</t>
-  </si>
-  <si>
     <t>C</t>
-  </si>
-  <si>
-    <t>IdCarpetaReportes</t>
-  </si>
-  <si>
-    <t>1i32WDbFZOhjmaND-ySCiCkkLQsiXoBQr</t>
   </si>
 </sst>
 </file>
@@ -1641,13 +1641,13 @@
         <v>123</v>
       </c>
       <c r="B3" s="25" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C3" s="26" t="s">
         <v>128</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1">
@@ -1672,10 +1672,10 @@
     </row>
     <row r="6" spans="1:26" ht="14.5">
       <c r="A6" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>227</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>228</v>
       </c>
     </row>
     <row r="7" spans="1:26" ht="14.25" customHeight="1">
@@ -1755,7 +1755,7 @@
         <v>142</v>
       </c>
       <c r="B13" t="s">
-        <v>224</v>
+        <v>252</v>
       </c>
     </row>
     <row r="14" spans="1:26" ht="14" customHeight="1">
@@ -1763,7 +1763,7 @@
         <v>143</v>
       </c>
       <c r="B14" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="15" spans="1:26" ht="14.25" customHeight="1">
@@ -2348,7 +2348,7 @@
         <v>102</v>
       </c>
       <c r="B84" s="39" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C84" s="39" t="s">
         <v>172</v>
@@ -2356,32 +2356,32 @@
     </row>
     <row r="85" spans="1:3" ht="14.25" customHeight="1">
       <c r="A85" s="52" t="s">
+        <v>229</v>
+      </c>
+      <c r="B85" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="C85" s="2" t="s">
         <v>230</v>
-      </c>
-      <c r="B85" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="C85" s="2" t="s">
-        <v>231</v>
       </c>
     </row>
     <row r="86" spans="1:3" ht="14.25" customHeight="1">
       <c r="A86" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="B86" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="C86" s="2" t="s">
         <v>235</v>
-      </c>
-      <c r="B86" s="2" t="s">
-        <v>250</v>
-      </c>
-      <c r="C86" s="2" t="s">
-        <v>236</v>
       </c>
     </row>
     <row r="87" spans="1:3" ht="14.25" customHeight="1">
       <c r="A87" s="52" t="s">
+        <v>231</v>
+      </c>
+      <c r="B87" s="2" t="s">
         <v>232</v>
-      </c>
-      <c r="B87" s="2" t="s">
-        <v>233</v>
       </c>
       <c r="C87" s="2"/>
     </row>
@@ -2443,48 +2443,48 @@
     </row>
     <row r="96" spans="1:3" ht="14.25" customHeight="1">
       <c r="A96" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="B96" s="2" t="s">
         <v>237</v>
-      </c>
-      <c r="B96" s="2" t="s">
-        <v>238</v>
       </c>
     </row>
     <row r="97" spans="1:3" ht="14.25" customHeight="1">
       <c r="A97" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="B97" t="s">
         <v>239</v>
-      </c>
-      <c r="B97" t="s">
-        <v>240</v>
       </c>
     </row>
     <row r="98" spans="1:3" ht="14.25" customHeight="1">
       <c r="A98" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="B98" t="s">
         <v>244</v>
       </c>
-      <c r="B98" t="s">
+      <c r="C98" s="2" t="s">
         <v>245</v>
-      </c>
-      <c r="C98" s="2" t="s">
-        <v>246</v>
       </c>
     </row>
     <row r="99" spans="1:3" ht="14.25" customHeight="1">
       <c r="A99" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="B99" t="s">
         <v>247</v>
       </c>
-      <c r="B99" t="s">
+      <c r="C99" s="2" t="s">
         <v>248</v>
-      </c>
-      <c r="C99" s="2" t="s">
-        <v>249</v>
       </c>
     </row>
     <row r="100" spans="1:3" ht="14.25" customHeight="1">
       <c r="A100" s="2" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="B100" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
     </row>
     <row r="101" spans="1:3" ht="14.25" customHeight="1"/>
@@ -5872,18 +5872,18 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="2" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="2" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B4" s="53" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Version del proyecto al dia 5 de octubre de 2026
</commit_message>
<xml_diff>
--- a/Archivos/CONFIGURACION/Config.xlsx
+++ b/Archivos/CONFIGURACION/Config.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Procesos_Uipath\541_DISPOINFOMEDALIABRYAM_NF_SEG_SEG\Archivos\CONFIGURACION\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BF18854-130B-4024-B638-4DD9C075DB85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99C650BE-809C-41FB-9136-93A219C086AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -813,94 +813,94 @@
     <t>END POINTS PARA MODULO "CHAT_RPA"</t>
   </si>
   <si>
+    <t>541_DISPOINFOMEDALIABRYAM_NF_SEG_SEG</t>
+  </si>
+  <si>
+    <t>Descargas</t>
+  </si>
+  <si>
+    <t>Downloads\</t>
+  </si>
+  <si>
+    <t>0AHVIhGN0elUOUk9PVA</t>
+  </si>
+  <si>
+    <t>Id_Template_Liverpool</t>
+  </si>
+  <si>
+    <t>Template de Google Sheet de Liverpool</t>
+  </si>
+  <si>
+    <t>Id_Carpeta_Config_Bot</t>
+  </si>
+  <si>
+    <t>1MW2qJxEnyfY3t5gfL9MOCKiYjNtK1CNp</t>
+  </si>
+  <si>
+    <t>1ZUrDKGkjrHELaHsYlGOsv9Sxd8xapjPZQoTOnLnCYZQ</t>
+  </si>
+  <si>
+    <t>Id_Template_Suburbia</t>
+  </si>
+  <si>
+    <t>Template de Google Sheet de Suburbia</t>
+  </si>
+  <si>
+    <t>Id_Sheet_PlantillaRegistrosGlobales</t>
+  </si>
+  <si>
+    <t>1Ho4_5n3e3SyFwS-abRHqeLuCXK__oC4Sz74XjNLceSk</t>
+  </si>
+  <si>
+    <t>Id_Sheet_FolderReportesDiarios</t>
+  </si>
+  <si>
+    <t>15dkrlT8OO6PJwchlXyckIVZmWdjoCbpE</t>
+  </si>
+  <si>
+    <t>Cred_Medallia</t>
+  </si>
+  <si>
+    <t>Usr_Active_Directory</t>
+  </si>
+  <si>
+    <t>Cred_Generica</t>
+  </si>
+  <si>
+    <t>IdSheetReprocesos</t>
+  </si>
+  <si>
+    <t>1LadTK_nCaO-3Den47XRLUp_ODoGlwgsBnScrscPbx0M</t>
+  </si>
+  <si>
+    <t>Archivo que determina las ejecuciones</t>
+  </si>
+  <si>
+    <t>IdSheetCorreosEnviados</t>
+  </si>
+  <si>
+    <t>1Bt8YI2hz2viYufv1tQpBy8gFyQR-RiKS</t>
+  </si>
+  <si>
+    <t>Folder para guardar historicos de correos enviados.</t>
+  </si>
+  <si>
+    <t>1aIFFCmYWICxlWv_rqnVRtiX2G4vyAWygaUnZZPSuwYE</t>
+  </si>
+  <si>
+    <t>IdCarpetaReportes</t>
+  </si>
+  <si>
+    <t>1i32WDbFZOhjmaND-ySCiCkkLQsiXoBQr</t>
+  </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>C:\Users\USR\AppData\Local\Programs\Python\Python38\</t>
+  </si>
+  <si>
     <t>C:\Program Files\Python38\</t>
-  </si>
-  <si>
-    <t>541_DISPOINFOMEDALIABRYAM_NF_SEG_SEG</t>
-  </si>
-  <si>
-    <t>Descargas</t>
-  </si>
-  <si>
-    <t>Downloads\</t>
-  </si>
-  <si>
-    <t>0AHVIhGN0elUOUk9PVA</t>
-  </si>
-  <si>
-    <t>Id_Template_Liverpool</t>
-  </si>
-  <si>
-    <t>Template de Google Sheet de Liverpool</t>
-  </si>
-  <si>
-    <t>Id_Carpeta_Config_Bot</t>
-  </si>
-  <si>
-    <t>1MW2qJxEnyfY3t5gfL9MOCKiYjNtK1CNp</t>
-  </si>
-  <si>
-    <t>1ZUrDKGkjrHELaHsYlGOsv9Sxd8xapjPZQoTOnLnCYZQ</t>
-  </si>
-  <si>
-    <t>Id_Template_Suburbia</t>
-  </si>
-  <si>
-    <t>Template de Google Sheet de Suburbia</t>
-  </si>
-  <si>
-    <t>Id_Sheet_PlantillaRegistrosGlobales</t>
-  </si>
-  <si>
-    <t>1Ho4_5n3e3SyFwS-abRHqeLuCXK__oC4Sz74XjNLceSk</t>
-  </si>
-  <si>
-    <t>Id_Sheet_FolderReportesDiarios</t>
-  </si>
-  <si>
-    <t>15dkrlT8OO6PJwchlXyckIVZmWdjoCbpE</t>
-  </si>
-  <si>
-    <t>Cred_Medallia</t>
-  </si>
-  <si>
-    <t>Usr_Active_Directory</t>
-  </si>
-  <si>
-    <t>Cred_Generica</t>
-  </si>
-  <si>
-    <t>IdSheetReprocesos</t>
-  </si>
-  <si>
-    <t>1LadTK_nCaO-3Den47XRLUp_ODoGlwgsBnScrscPbx0M</t>
-  </si>
-  <si>
-    <t>Archivo que determina las ejecuciones</t>
-  </si>
-  <si>
-    <t>IdSheetCorreosEnviados</t>
-  </si>
-  <si>
-    <t>1Bt8YI2hz2viYufv1tQpBy8gFyQR-RiKS</t>
-  </si>
-  <si>
-    <t>Folder para guardar historicos de correos enviados.</t>
-  </si>
-  <si>
-    <t>1aIFFCmYWICxlWv_rqnVRtiX2G4vyAWygaUnZZPSuwYE</t>
-  </si>
-  <si>
-    <t>IdCarpetaReportes</t>
-  </si>
-  <si>
-    <t>1i32WDbFZOhjmaND-ySCiCkkLQsiXoBQr</t>
-  </si>
-  <si>
-    <t>C:\Users\USR\AppData\Local\Programs\Python\Python38\</t>
-  </si>
-  <si>
-    <t>C</t>
   </si>
 </sst>
 </file>
@@ -1641,13 +1641,13 @@
         <v>123</v>
       </c>
       <c r="B3" s="25" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C3" s="26" t="s">
         <v>128</v>
       </c>
-      <c r="E3" s="2" t="s">
-        <v>253</v>
+      <c r="E3" t="s">
+        <v>251</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1">
@@ -1672,10 +1672,10 @@
     </row>
     <row r="6" spans="1:26" ht="14.5">
       <c r="A6" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>226</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>227</v>
       </c>
     </row>
     <row r="7" spans="1:26" ht="14.25" customHeight="1">
@@ -1684,7 +1684,7 @@
       </c>
       <c r="B7" s="2" t="str">
         <f>_xlfn.CONCAT($E$3, ":\Procesos_UiPath\"&amp;B3&amp;"\Archivos\")</f>
-        <v>C:\Procesos_UiPath\541_DISPOINFOMEDALIABRYAM_NF_SEG_SEG\Archivos\</v>
+        <v>D:\Procesos_UiPath\541_DISPOINFOMEDALIABRYAM_NF_SEG_SEG\Archivos\</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>133</v>
@@ -1696,7 +1696,7 @@
       </c>
       <c r="B8" s="2" t="str">
         <f>_xlfn.CONCAT($E$3, ":\Procesos_UiPath\"&amp;B3&amp;"\Archivos\"&amp;B4&amp;"\")</f>
-        <v>C:\Procesos_UiPath\541_DISPOINFOMEDALIABRYAM_NF_SEG_SEG\Archivos\Temporal\</v>
+        <v>D:\Procesos_UiPath\541_DISPOINFOMEDALIABRYAM_NF_SEG_SEG\Archivos\Temporal\</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>134</v>
@@ -1708,7 +1708,7 @@
       </c>
       <c r="B9" s="2" t="str">
         <f>_xlfn.CONCAT($E$3, ":\Procesos_UiPath\"&amp;B3&amp;"\Archivos\"&amp;B4&amp;"_Error")</f>
-        <v>C:\Procesos_UiPath\541_DISPOINFOMEDALIABRYAM_NF_SEG_SEG\Archivos\Temporal_Error</v>
+        <v>D:\Procesos_UiPath\541_DISPOINFOMEDALIABRYAM_NF_SEG_SEG\Archivos\Temporal_Error</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>136</v>
@@ -1720,7 +1720,7 @@
       </c>
       <c r="B10" t="str">
         <f>_xlfn.CONCAT($E$3, ":\Procesos_UiPath\"&amp;B3&amp;"\Archivos\FORMATOS\")</f>
-        <v>C:\Procesos_UiPath\541_DISPOINFOMEDALIABRYAM_NF_SEG_SEG\Archivos\FORMATOS\</v>
+        <v>D:\Procesos_UiPath\541_DISPOINFOMEDALIABRYAM_NF_SEG_SEG\Archivos\FORMATOS\</v>
       </c>
       <c r="C10" t="s">
         <v>137</v>
@@ -1732,7 +1732,7 @@
       </c>
       <c r="B11" s="2" t="str">
         <f>_xlfn.CONCAT($E$3, ":\Procesos_UiPath\"&amp;B3&amp;"\Archivos\CONFIGURACION\")</f>
-        <v>C:\Procesos_UiPath\541_DISPOINFOMEDALIABRYAM_NF_SEG_SEG\Archivos\CONFIGURACION\</v>
+        <v>D:\Procesos_UiPath\541_DISPOINFOMEDALIABRYAM_NF_SEG_SEG\Archivos\CONFIGURACION\</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>139</v>
@@ -1744,7 +1744,7 @@
       </c>
       <c r="B12" s="2" t="str">
         <f>_xlfn.CONCAT($E$3, ":\Procesos_UiPath\"&amp;B3&amp;"\Archivos\Exceptions_Screenshots\")</f>
-        <v>C:\Procesos_UiPath\541_DISPOINFOMEDALIABRYAM_NF_SEG_SEG\Archivos\Exceptions_Screenshots\</v>
+        <v>D:\Procesos_UiPath\541_DISPOINFOMEDALIABRYAM_NF_SEG_SEG\Archivos\Exceptions_Screenshots\</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>141</v>
@@ -1763,7 +1763,7 @@
         <v>143</v>
       </c>
       <c r="B14" t="s">
-        <v>224</v>
+        <v>253</v>
       </c>
     </row>
     <row r="15" spans="1:26" ht="14.25" customHeight="1">
@@ -2348,7 +2348,7 @@
         <v>102</v>
       </c>
       <c r="B84" s="39" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C84" s="39" t="s">
         <v>172</v>
@@ -2356,32 +2356,32 @@
     </row>
     <row r="85" spans="1:3" ht="14.25" customHeight="1">
       <c r="A85" s="52" t="s">
+        <v>228</v>
+      </c>
+      <c r="B85" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="C85" s="2" t="s">
         <v>229</v>
-      </c>
-      <c r="B85" s="2" t="s">
-        <v>233</v>
-      </c>
-      <c r="C85" s="2" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="86" spans="1:3" ht="14.25" customHeight="1">
       <c r="A86" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="B86" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="C86" s="2" t="s">
         <v>234</v>
-      </c>
-      <c r="B86" s="2" t="s">
-        <v>249</v>
-      </c>
-      <c r="C86" s="2" t="s">
-        <v>235</v>
       </c>
     </row>
     <row r="87" spans="1:3" ht="14.25" customHeight="1">
       <c r="A87" s="52" t="s">
+        <v>230</v>
+      </c>
+      <c r="B87" s="2" t="s">
         <v>231</v>
-      </c>
-      <c r="B87" s="2" t="s">
-        <v>232</v>
       </c>
       <c r="C87" s="2"/>
     </row>
@@ -2391,7 +2391,7 @@
       </c>
       <c r="B88" s="41" t="str">
         <f>_xlfn.CONCAT(E3,":\Procesos_UiPath\Llaves\crp-pro-ccoe-automat-c9c501f57fdd_NF.json")</f>
-        <v>C:\Procesos_UiPath\Llaves\crp-pro-ccoe-automat-c9c501f57fdd_NF.json</v>
+        <v>D:\Procesos_UiPath\Llaves\crp-pro-ccoe-automat-c9c501f57fdd_NF.json</v>
       </c>
       <c r="C88" s="42" t="s">
         <v>124</v>
@@ -2443,48 +2443,48 @@
     </row>
     <row r="96" spans="1:3" ht="14.25" customHeight="1">
       <c r="A96" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="B96" s="2" t="s">
         <v>236</v>
-      </c>
-      <c r="B96" s="2" t="s">
-        <v>237</v>
       </c>
     </row>
     <row r="97" spans="1:3" ht="14.25" customHeight="1">
       <c r="A97" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="B97" t="s">
         <v>238</v>
-      </c>
-      <c r="B97" t="s">
-        <v>239</v>
       </c>
     </row>
     <row r="98" spans="1:3" ht="14.25" customHeight="1">
       <c r="A98" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="B98" t="s">
         <v>243</v>
       </c>
-      <c r="B98" t="s">
+      <c r="C98" s="2" t="s">
         <v>244</v>
-      </c>
-      <c r="C98" s="2" t="s">
-        <v>245</v>
       </c>
     </row>
     <row r="99" spans="1:3" ht="14.25" customHeight="1">
       <c r="A99" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="B99" t="s">
         <v>246</v>
       </c>
-      <c r="B99" t="s">
+      <c r="C99" s="2" t="s">
         <v>247</v>
-      </c>
-      <c r="C99" s="2" t="s">
-        <v>248</v>
       </c>
     </row>
     <row r="100" spans="1:3" ht="14.25" customHeight="1">
       <c r="A100" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="B100" t="s">
         <v>250</v>
-      </c>
-      <c r="B100" t="s">
-        <v>251</v>
       </c>
     </row>
     <row r="101" spans="1:3" ht="14.25" customHeight="1"/>
@@ -5872,18 +5872,18 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="2" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="2" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B4" s="53" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
   </sheetData>

</xml_diff>